<commit_message>
Fase 3: ALV, BAPI BP, commit/rollback, log
</commit_message>
<xml_diff>
--- a/Proyecto Final Desarrollo ABAP con COPILOT.xlsx
+++ b/Proyecto Final Desarrollo ABAP con COPILOT.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\FranciscoValenzuela\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://icasa365-my.sharepoint.com/personal/franciscovalenzuela_icasa_com_gt/Documents/Proyecto Final Copilot/Proyecto Final/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED211023-8865-4406-8627-7D9DA1F88976}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{ED211023-8865-4406-8627-7D9DA1F88976}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2AFBA6D5-8D4E-4DBA-AB0C-431479055EF8}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{90EE437F-81CB-4A4E-AE2C-0A8773015A8E}"/>
   </bookViews>
@@ -861,6 +861,9 @@
       <c r="C24">
         <v>2.5</v>
       </c>
+      <c r="D24">
+        <v>1.5</v>
+      </c>
       <c r="E24" t="s">
         <v>15</v>
       </c>
@@ -872,6 +875,9 @@
       <c r="C25">
         <v>4</v>
       </c>
+      <c r="D25">
+        <v>2.5</v>
+      </c>
       <c r="E25" t="s">
         <v>15</v>
       </c>
@@ -883,6 +889,9 @@
       <c r="C26">
         <v>2.5</v>
       </c>
+      <c r="D26">
+        <v>1.5</v>
+      </c>
       <c r="E26" t="s">
         <v>15</v>
       </c>
@@ -894,6 +903,9 @@
       <c r="C27">
         <v>5</v>
       </c>
+      <c r="D27">
+        <v>3.5</v>
+      </c>
       <c r="E27" t="s">
         <v>15</v>
       </c>
@@ -905,6 +917,9 @@
       <c r="C28">
         <v>2</v>
       </c>
+      <c r="D28">
+        <v>1</v>
+      </c>
       <c r="E28" t="s">
         <v>15</v>
       </c>
@@ -916,6 +931,9 @@
       <c r="C29">
         <v>3</v>
       </c>
+      <c r="D29">
+        <v>2</v>
+      </c>
       <c r="E29" t="s">
         <v>15</v>
       </c>
@@ -930,7 +948,7 @@
       </c>
       <c r="D31">
         <f>SUM(D24:D30)</f>
-        <v>0</v>
+        <v>12</v>
       </c>
     </row>
     <row r="32" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1075,7 +1093,7 @@
       </c>
       <c r="D48">
         <f>SUM(D12,D22,D31,D39,D47)</f>
-        <v>20.5</v>
+        <v>32.5</v>
       </c>
     </row>
     <row r="49" spans="2:4" x14ac:dyDescent="0.25">
@@ -1088,7 +1106,7 @@
       </c>
       <c r="D49" s="5">
         <f>D48/40</f>
-        <v>0.51249999999999996</v>
+        <v>0.8125</v>
       </c>
     </row>
     <row r="50" spans="2:4" x14ac:dyDescent="0.25">
@@ -1101,7 +1119,7 @@
       </c>
       <c r="D50" s="5">
         <f>D48/8</f>
-        <v>2.5625</v>
+        <v>4.0625</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualiza Excel: Fase 4 (horas Copilot)
Se ajusta la planificación de Fase 4 agregando desglose de horas Copilot vs manual por actividad.
</commit_message>
<xml_diff>
--- a/Proyecto Final Desarrollo ABAP con COPILOT.xlsx
+++ b/Proyecto Final Desarrollo ABAP con COPILOT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://icasa365-my.sharepoint.com/personal/franciscovalenzuela_icasa_com_gt/Documents/Proyecto Final Copilot/Proyecto Final/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{ED211023-8865-4406-8627-7D9DA1F88976}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2AFBA6D5-8D4E-4DBA-AB0C-431479055EF8}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="13_ncr:1_{ED211023-8865-4406-8627-7D9DA1F88976}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B903F1FC-AC87-4FDC-AF13-4FF7BD99B918}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{90EE437F-81CB-4A4E-AE2C-0A8773015A8E}"/>
   </bookViews>
@@ -963,6 +963,9 @@
       <c r="C33">
         <v>2</v>
       </c>
+      <c r="D33">
+        <v>1</v>
+      </c>
       <c r="E33" t="s">
         <v>15</v>
       </c>
@@ -974,6 +977,9 @@
       <c r="C34">
         <v>2</v>
       </c>
+      <c r="D34">
+        <v>1</v>
+      </c>
       <c r="E34" t="s">
         <v>15</v>
       </c>
@@ -985,6 +991,9 @@
       <c r="C35">
         <v>2.5</v>
       </c>
+      <c r="D35">
+        <v>1.2</v>
+      </c>
       <c r="E35" t="s">
         <v>15</v>
       </c>
@@ -996,6 +1005,9 @@
       <c r="C36">
         <v>3</v>
       </c>
+      <c r="D36">
+        <v>2</v>
+      </c>
       <c r="E36" t="s">
         <v>15</v>
       </c>
@@ -1007,6 +1019,9 @@
       <c r="C37">
         <v>2</v>
       </c>
+      <c r="D37">
+        <v>1</v>
+      </c>
       <c r="E37" t="s">
         <v>15</v>
       </c>
@@ -1021,7 +1036,7 @@
       </c>
       <c r="D39">
         <f>SUM(D33:D38)</f>
-        <v>0</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="41" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1036,6 +1051,9 @@
       <c r="C42">
         <v>3</v>
       </c>
+      <c r="D42">
+        <v>1.5</v>
+      </c>
       <c r="E42" t="s">
         <v>15</v>
       </c>
@@ -1047,6 +1065,9 @@
       <c r="C43">
         <v>3</v>
       </c>
+      <c r="D43">
+        <v>1.5</v>
+      </c>
       <c r="E43" t="s">
         <v>15</v>
       </c>
@@ -1058,6 +1079,9 @@
       <c r="C44">
         <v>2.5</v>
       </c>
+      <c r="D44">
+        <v>1</v>
+      </c>
       <c r="E44" t="s">
         <v>15</v>
       </c>
@@ -1068,6 +1092,9 @@
       </c>
       <c r="C45">
         <v>2</v>
+      </c>
+      <c r="D45">
+        <v>1</v>
       </c>
       <c r="E45" t="s">
         <v>15</v>
@@ -1080,7 +1107,7 @@
       </c>
       <c r="D47">
         <f>SUM(D42:D46)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="48" spans="2:5" x14ac:dyDescent="0.25">
@@ -1093,7 +1120,7 @@
       </c>
       <c r="D48">
         <f>SUM(D12,D22,D31,D39,D47)</f>
-        <v>32.5</v>
+        <v>43.7</v>
       </c>
     </row>
     <row r="49" spans="2:4" x14ac:dyDescent="0.25">
@@ -1106,7 +1133,7 @@
       </c>
       <c r="D49" s="5">
         <f>D48/40</f>
-        <v>0.8125</v>
+        <v>1.0925</v>
       </c>
     </row>
     <row r="50" spans="2:4" x14ac:dyDescent="0.25">
@@ -1119,7 +1146,7 @@
       </c>
       <c r="D50" s="5">
         <f>D48/8</f>
-        <v>4.0625</v>
+        <v>5.4625000000000004</v>
       </c>
     </row>
   </sheetData>

</xml_diff>